<commit_message>
VR Projection, AV1 output, a runtime Image Size dial, and two silent-failure fixes that make long runs stable
</commit_message>
<xml_diff>
--- a/ChitraMaya-Roadmap.xlsx
+++ b/ChitraMaya-Roadmap.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyProjects\ChitraMaya\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gsada\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7049AB41-9744-47D1-8B6F-50F8B2DD183E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C883BD9-A9D9-4449-B3BC-8837A92C4DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Roadmap" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Roadmap!$A$1:$J$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Roadmap!$A$1:$J$76</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="264">
   <si>
     <t>ID</t>
   </si>
@@ -358,21 +358,21 @@
     <t>CM-029</t>
   </si>
   <si>
+    <t>Model Management window</t>
+  </si>
+  <si>
+    <t>Manage Models modal: source-URL dropdown (seeded with ladaapp + zelefans HF repos, learns user-added, persists to model-sources.json) -&gt; fetch via HF list_repo_files -&gt; multi-select picker -&gt; Compile, driving Compile-All-Engines.ps1 (CM-007) with the compile log streamed into a pane. v1 shells out to the PS1 (don't re-port hard-won compile flags). Last blocker for fresh installs (no engines shipped). https://huggingface.co/zelefans DONE (field-verified: download + compile on 5060Ti / 3060 12GB / 3060 6GB / 4060 8GB; the HF-403 download hardening is CM-060). Two corrections to the original spec: it drives the exe's -compile-det/-compile-rest subcommands directly (not the PS1 - same flags, no PowerShell dependency), and it is no longer a fresh-install blocker. Residual Manage-Models poll polish tracked as CM-065.</t>
+  </si>
+  <si>
+    <t>Roadmap</t>
+  </si>
+  <si>
+    <t>CM-030</t>
+  </si>
+  <si>
     <t>Open</t>
   </si>
   <si>
-    <t>Model Management window</t>
-  </si>
-  <si>
-    <t>Manage Models modal: source-URL dropdown (seeded with ladaapp + zelefans HF repos, learns user-added, persists to model-sources.json) -&gt; fetch via HF list_repo_files -&gt; multi-select picker -&gt; Compile, driving Compile-All-Engines.ps1 (CM-007) with the compile log streamed into a pane. v1 shells out to the PS1 (don't re-port hard-won compile flags). Last blocker for fresh installs (no engines shipped). https://huggingface.co/zelefans</t>
-  </si>
-  <si>
-    <t>Roadmap</t>
-  </si>
-  <si>
-    <t>CM-030</t>
-  </si>
-  <si>
     <t>GPU-arch detection + unsupported-GPU message</t>
   </si>
   <si>
@@ -692,6 +692,129 @@
   </si>
   <si>
     <t>Closing the console window kills the server (built console=True). Build console=False (windowed) + a Windows AttachConsole(parent) shim so CLI subcommands still stream to their terminal + a rotating log file, so a UI launch has no closable terminal to kill by accident. Needs packaged-build testing. From CM-049.</t>
+  </si>
+  <si>
+    <t>CM-065</t>
+  </si>
+  <si>
+    <t>Manage Models poll-lifecycle fixes</t>
+  </si>
+  <si>
+    <t>Two Manage-Models UI bugs from CM-049. (1) closeManageModels() cleared only the compile poll (_mmPoll), not the download poll (_mmDlPoll) - a download poll kept firing every 800ms against the hidden modal after close; now clears BOTH. (2) Compile and download share the single #mmLog pane (and the GPU): extracted _mmStartDlPolling() so a running download resumes on reopen (was: only compile resumed), and added a guard so the two can't run concurrently (their logs would overwrite each other tick-by-tick). Fix Batch 8.</t>
+  </si>
+  <si>
+    <t>CM-066</t>
+  </si>
+  <si>
+    <t>SBS</t>
+  </si>
+  <si>
+    <t>SBS View - projected 3D compare viewer</t>
+  </si>
+  <si>
+    <t>Projected equirect-180 per-eye viewer on the main player (SBS button): drag look-around + wheel zoom, Eye L/R, View Original/Restored/Wipe with draggable divider, frame-locked A/B sync (playbackRate-nudge; hard-seek only on jumps), full transport with frame stepping + app skip amounts, 0.1-1x speed, segment-preview clock offset, Esc frees decoders. three.js r185 vendored (module+core). Shipped v1.10.00 (Batch 10 + transport/view/sync drops).</t>
+  </si>
+  <si>
+    <t>Gman + Claude</t>
+  </si>
+  <si>
+    <t>CM-067</t>
+  </si>
+  <si>
+    <t>Add Mosaic (manual) - draw rectangles + pixelate (SFW censor)</t>
+  </si>
+  <si>
+    <t>Pixelate up to 3 regions and save (-mosaic.mp4 / -mosaic-seg.mp4). Draw layer on the paused player (object-fit-exact mapping, size labels, x delete, banner Done/Type/Cancel), per-eye SBS coords auto-mirrored with live dashed ghost, dialog pre-filled for numeric fine-tune, Draw again keeps rects. gRestorer pixelate kernel on ChitraMaya Decoder/Encoder. Output becomes preview so SBS View wipe-verifies. Shipped v1.10.00 (Batches 11-12 + New/button-state fixes).</t>
+  </si>
+  <si>
+    <t>CM-068</t>
+  </si>
+  <si>
+    <t>Manage Models modal overflow on long lists (issue #3) + Esc close</t>
+  </si>
+  <si>
+    <t>First external bug: long fetched model list pushed Close off-screen (1080p and up). Modal now flex column capped 90vh, title+Close pinned, body scrolls; base .modal gets 90vh/overflow safety net for all modals; Esc closes (jobs keep running server-side, resume on reopen). Verified headless at exactly 1920x1080 with 40+30-row lists. Shipped v1.20.00 (Batch 13).</t>
+  </si>
+  <si>
+    <t>GitHub issue #3</t>
+  </si>
+  <si>
+    <t>https://github.com/seatv/ChitraMaya/issues/3</t>
+  </si>
+  <si>
+    <t>CM-069</t>
+  </si>
+  <si>
+    <t>Single-source version constant</t>
+  </si>
+  <si>
+    <t>chitramaya/__init__.py __version__ is the one line bumped per release; HF download User-Agent (ChitraMaya/&lt;ver&gt;) and window title read it. Replaced stale hardcoded UA. Shipped v1.20.00 (Batch 14).</t>
+  </si>
+  <si>
+    <t>CM-070</t>
+  </si>
+  <si>
+    <t>Auto Mosaic - NSFW-detection censor mode (EXPERIMENTAL)</t>
+  </si>
+  <si>
+    <t>Detect-and-pixelate via pluggable MosaicClipRestorer (mode=mosaic): reuses full detect/track/SBS/composite path, no restoration model needed. Surfaced as Alternate Execution Modes (Add Mosaic + Block, mutually exclusive with renamed Preview Detection) so Test Frame (Original-&gt;Censored), Restore and Restore &amp; Save all honor it; one-shot Auto-detect in the dialog; output -censored.mp4. Field verdict: mechanics solid, lada NSFW model v1.3 (YOLO-seg, 1 class, 640) misses frames - NOT production censoring; documented experimental in README/T&amp;C/notes. Shipped v1.20.00 (Batches 14-15).</t>
+  </si>
+  <si>
+    <t>CM-071</t>
+  </si>
+  <si>
+    <t>Playback speed control on main player</t>
+  </si>
+  <si>
+    <t>Slider + readout left of SBS button; 14 multiplicative steps 0.0625x-16x (full WebView2 range), double-click resets 1x, persists across original&lt;-&gt;preview src swaps (loadedmetadata reapply). For spotting missed mosaic frames (slow) and skimming (fast). Shipped v1.20.00 (Batch 16).</t>
+  </si>
+  <si>
+    <t>Gman request</t>
+  </si>
+  <si>
+    <t>CM-072</t>
+  </si>
+  <si>
+    <t>Evaluate FaceFusion NSFW detectors as Auto Mosaic backends</t>
+  </si>
+  <si>
+    <t>lada NSFW model misses frames and author is unreachable. FaceFusion runs three NSFW detectors (content-analyser); evaluate what each returns (class/box/mask? video-capable?), licensing, and whether any can slot into the YOLO-seg detection path or needs an adapter. Goal: raise Auto Mosaic recall toward production-usable censoring.</t>
+  </si>
+  <si>
+    <t>Gman (v1.20 verdict)</t>
+  </si>
+  <si>
+    <t>CM-073</t>
+  </si>
+  <si>
+    <t>Player error toast for undecodable files</t>
+  </si>
+  <si>
+    <t>Main player &lt;video&gt; fails silently (no error listener) on anything WebView2 cannot decode - stray .ts, HEVC without OS extensions, odd containers - shows dead Play button. Add player error handler with plain-language toast (what happened + that restoration still works + likely fix). Papercut found via .ts false alarm; also queued in Batch 13 notes.</t>
+  </si>
+  <si>
+    <t>Field testing</t>
+  </si>
+  <si>
+    <t>CM-074</t>
+  </si>
+  <si>
+    <t>SBS View projection selector (fisheye 190/200)</t>
+  </si>
+  <si>
+    <t>Viewer assumes equirect-180 LR; fisheye VR sources project wrong. Add a projection dropdown - swap is confined to the direction-&gt;UV function in the fragment shader. Documented as known limitation in v1.10/v1.20 notes.</t>
+  </si>
+  <si>
+    <t>SBS viewer plan</t>
+  </si>
+  <si>
+    <t>CM-075</t>
+  </si>
+  <si>
+    <t>AV1 (NVENC) encoding support</t>
+  </si>
+  <si>
+    <t>Add av1 to the encoder codec choices (UI Encoder dropdown + --enc-codec). HARDWARE GATE: NVENC AV1 encode requires Ada (RTX 40-series) or Blackwell (50-series); Ampere 30-series cannot encode AV1 (it CAN decode via NVDEC). Work: PyNvVideoCodec AV1 encode session + settings mapping (preset/QP; bf/profile differ from HEVC), capability probe with clear unsupported-GPU error naming the fix (choose hevc/h264), remux with av01 tag + faststart, verify A/V sync path. Bonus: Chromium/WebView2 decodes AV1 natively - previews and SBS View work with NO HEVC extensions dependency. Fleet: 5060Ti + 4060 can encode; 3060s validate decode-only path. ~30% bitrate savings vs HEVC at same quality for 8K VR distribution.</t>
   </si>
 </sst>
 </file>
@@ -1040,7 +1163,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J65"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1087,7 +1211,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45">
+    <row r="2" spans="1:10" ht="45" hidden="1">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1115,7 +1239,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" ht="30">
+    <row r="3" spans="1:10" ht="30" hidden="1">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -1143,7 +1267,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" ht="60">
+    <row r="4" spans="1:10" ht="60" hidden="1">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -1171,7 +1295,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="45">
+    <row r="5" spans="1:10" ht="45" hidden="1">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -1199,7 +1323,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" ht="45">
+    <row r="6" spans="1:10" ht="45" hidden="1">
       <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
@@ -1227,7 +1351,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" ht="45">
+    <row r="7" spans="1:10" ht="45" hidden="1">
       <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1255,7 +1379,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" ht="45">
+    <row r="8" spans="1:10" ht="45" hidden="1">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -1283,7 +1407,7 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10" ht="30">
+    <row r="9" spans="1:10" ht="30" hidden="1">
       <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
@@ -1311,7 +1435,7 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10" ht="30">
+    <row r="10" spans="1:10" ht="30" hidden="1">
       <c r="A10" s="1" t="s">
         <v>42</v>
       </c>
@@ -1339,7 +1463,7 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="1:10" ht="45">
+    <row r="11" spans="1:10" ht="45" hidden="1">
       <c r="A11" s="1" t="s">
         <v>45</v>
       </c>
@@ -1367,7 +1491,7 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="1:10" ht="45">
+    <row r="12" spans="1:10" ht="45" hidden="1">
       <c r="A12" s="1" t="s">
         <v>49</v>
       </c>
@@ -1395,7 +1519,7 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:10" ht="45">
+    <row r="13" spans="1:10" ht="45" hidden="1">
       <c r="A13" s="1" t="s">
         <v>52</v>
       </c>
@@ -1423,7 +1547,7 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:10" ht="45">
+    <row r="14" spans="1:10" ht="45" hidden="1">
       <c r="A14" s="1" t="s">
         <v>56</v>
       </c>
@@ -1451,7 +1575,7 @@
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="1:10" ht="75">
+    <row r="15" spans="1:10" ht="75" hidden="1">
       <c r="A15" s="1" t="s">
         <v>59</v>
       </c>
@@ -1479,7 +1603,7 @@
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="1:10" ht="60">
+    <row r="16" spans="1:10" ht="60" hidden="1">
       <c r="A16" s="1" t="s">
         <v>63</v>
       </c>
@@ -1507,7 +1631,7 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="60">
+    <row r="17" spans="1:10" ht="60" hidden="1">
       <c r="A17" s="1" t="s">
         <v>66</v>
       </c>
@@ -1535,7 +1659,7 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:10" ht="60">
+    <row r="18" spans="1:10" ht="60" hidden="1">
       <c r="A18" s="1" t="s">
         <v>69</v>
       </c>
@@ -1563,7 +1687,7 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="1:10" ht="75">
+    <row r="19" spans="1:10" ht="75" hidden="1">
       <c r="A19" s="1" t="s">
         <v>74</v>
       </c>
@@ -1591,7 +1715,7 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="1:10" ht="75">
+    <row r="20" spans="1:10" ht="75" hidden="1">
       <c r="A20" s="1" t="s">
         <v>78</v>
       </c>
@@ -1619,7 +1743,7 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" spans="1:10" ht="60">
+    <row r="21" spans="1:10" ht="60" hidden="1">
       <c r="A21" s="1" t="s">
         <v>81</v>
       </c>
@@ -1647,7 +1771,7 @@
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
     </row>
-    <row r="22" spans="1:10" ht="60">
+    <row r="22" spans="1:10" ht="60" hidden="1">
       <c r="A22" s="1" t="s">
         <v>84</v>
       </c>
@@ -1675,7 +1799,7 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
     </row>
-    <row r="23" spans="1:10" ht="60">
+    <row r="23" spans="1:10" ht="60" hidden="1">
       <c r="A23" s="1" t="s">
         <v>87</v>
       </c>
@@ -1703,7 +1827,7 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
     </row>
-    <row r="24" spans="1:10" ht="60">
+    <row r="24" spans="1:10" ht="60" hidden="1">
       <c r="A24" s="1" t="s">
         <v>90</v>
       </c>
@@ -1731,7 +1855,7 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
     </row>
-    <row r="25" spans="1:10" ht="75">
+    <row r="25" spans="1:10" ht="75" hidden="1">
       <c r="A25" s="1" t="s">
         <v>94</v>
       </c>
@@ -1759,7 +1883,7 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="75">
+    <row r="26" spans="1:10" ht="75" hidden="1">
       <c r="A26" s="1" t="s">
         <v>98</v>
       </c>
@@ -1787,7 +1911,7 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
     </row>
-    <row r="27" spans="1:10" ht="75">
+    <row r="27" spans="1:10" ht="75" hidden="1">
       <c r="A27" s="1" t="s">
         <v>101</v>
       </c>
@@ -1815,7 +1939,7 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
     </row>
-    <row r="28" spans="1:10" ht="45">
+    <row r="28" spans="1:10" ht="45" hidden="1">
       <c r="A28" s="1" t="s">
         <v>104</v>
       </c>
@@ -1843,7 +1967,7 @@
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
     </row>
-    <row r="29" spans="1:10" ht="30">
+    <row r="29" spans="1:10" ht="30" hidden="1">
       <c r="A29" s="1" t="s">
         <v>107</v>
       </c>
@@ -1871,7 +1995,7 @@
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
     </row>
-    <row r="30" spans="1:10" ht="90">
+    <row r="30" spans="1:10" ht="165" hidden="1">
       <c r="A30" s="1" t="s">
         <v>110</v>
       </c>
@@ -1879,19 +2003,19 @@
         <v>28</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>111</v>
+        <v>12</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="G30" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="H30" s="3">
         <v>46212</v>
@@ -1901,13 +2025,13 @@
     </row>
     <row r="31" spans="1:10" ht="60">
       <c r="A31" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>32</v>
@@ -1919,7 +2043,7 @@
         <v>117</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H31" s="3">
         <v>46212</v>
@@ -1935,7 +2059,7 @@
         <v>28</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>91</v>
@@ -1963,7 +2087,7 @@
         <v>39</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>75</v>
@@ -1991,7 +2115,7 @@
         <v>39</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>91</v>
@@ -2019,7 +2143,7 @@
         <v>39</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>95</v>
@@ -2031,7 +2155,7 @@
         <v>129</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H35" s="3">
         <v>46212</v>
@@ -2047,7 +2171,7 @@
         <v>131</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>75</v>
@@ -2059,7 +2183,7 @@
         <v>133</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H36" s="3">
         <v>46212</v>
@@ -2067,7 +2191,7 @@
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
     </row>
-    <row r="37" spans="1:10" ht="105">
+    <row r="37" spans="1:10" ht="105" hidden="1">
       <c r="A37" s="1" t="s">
         <v>134</v>
       </c>
@@ -2087,7 +2211,7 @@
         <v>136</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H37" s="3">
         <v>46212</v>
@@ -2103,7 +2227,7 @@
         <v>39</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>13</v>
@@ -2131,7 +2255,7 @@
         <v>39</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>13</v>
@@ -2159,7 +2283,7 @@
         <v>131</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>13</v>
@@ -2187,7 +2311,7 @@
         <v>131</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>13</v>
@@ -2215,7 +2339,7 @@
         <v>39</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>70</v>
@@ -2243,7 +2367,7 @@
         <v>39</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>13</v>
@@ -2268,10 +2392,10 @@
         <v>155</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>70</v>
@@ -2296,10 +2420,10 @@
         <v>158</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>39</v>
+        <v>131</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>13</v>
@@ -2324,10 +2448,10 @@
         <v>161</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>13</v>
@@ -2352,10 +2476,10 @@
         <v>164</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>39</v>
+        <v>131</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>53</v>
@@ -2383,7 +2507,7 @@
         <v>131</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>32</v>
@@ -2411,7 +2535,7 @@
         <v>131</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>32</v>
@@ -2431,7 +2555,7 @@
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
     </row>
-    <row r="50" spans="1:10" ht="75">
+    <row r="50" spans="1:10" ht="75" hidden="1">
       <c r="A50" s="1" t="s">
         <v>173</v>
       </c>
@@ -2459,7 +2583,7 @@
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
     </row>
-    <row r="51" spans="1:10" ht="60">
+    <row r="51" spans="1:10" ht="60" hidden="1">
       <c r="A51" s="1" t="s">
         <v>177</v>
       </c>
@@ -2487,7 +2611,7 @@
       <c r="I51" s="1"/>
       <c r="J51" s="1"/>
     </row>
-    <row r="52" spans="1:10" ht="75">
+    <row r="52" spans="1:10" ht="75" hidden="1">
       <c r="A52" s="1" t="s">
         <v>180</v>
       </c>
@@ -2515,7 +2639,7 @@
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
     </row>
-    <row r="53" spans="1:10" ht="90">
+    <row r="53" spans="1:10" ht="90" hidden="1">
       <c r="A53" s="1" t="s">
         <v>183</v>
       </c>
@@ -2543,7 +2667,7 @@
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
     </row>
-    <row r="54" spans="1:10" ht="75">
+    <row r="54" spans="1:10" ht="75" hidden="1">
       <c r="A54" s="1" t="s">
         <v>187</v>
       </c>
@@ -2571,7 +2695,7 @@
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
     </row>
-    <row r="55" spans="1:10" ht="105">
+    <row r="55" spans="1:10" ht="105" hidden="1">
       <c r="A55" s="1" t="s">
         <v>190</v>
       </c>
@@ -2599,7 +2723,7 @@
       <c r="I55" s="1"/>
       <c r="J55" s="1"/>
     </row>
-    <row r="56" spans="1:10" ht="90">
+    <row r="56" spans="1:10" ht="90" hidden="1">
       <c r="A56" s="1" t="s">
         <v>193</v>
       </c>
@@ -2627,7 +2751,7 @@
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
     </row>
-    <row r="57" spans="1:10" ht="105">
+    <row r="57" spans="1:10" ht="105" hidden="1">
       <c r="A57" s="1" t="s">
         <v>196</v>
       </c>
@@ -2655,7 +2779,7 @@
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
     </row>
-    <row r="58" spans="1:10" ht="45">
+    <row r="58" spans="1:10" ht="45" hidden="1">
       <c r="A58" s="1" t="s">
         <v>199</v>
       </c>
@@ -2683,7 +2807,7 @@
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
     </row>
-    <row r="59" spans="1:10" ht="105">
+    <row r="59" spans="1:10" ht="105" hidden="1">
       <c r="A59" s="1" t="s">
         <v>202</v>
       </c>
@@ -2711,7 +2835,7 @@
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
     </row>
-    <row r="60" spans="1:10" ht="75">
+    <row r="60" spans="1:10" ht="75" hidden="1">
       <c r="A60" s="1" t="s">
         <v>205</v>
       </c>
@@ -2739,7 +2863,7 @@
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
     </row>
-    <row r="61" spans="1:10" ht="90">
+    <row r="61" spans="1:10" ht="90" hidden="1">
       <c r="A61" s="1" t="s">
         <v>208</v>
       </c>
@@ -2775,7 +2899,7 @@
         <v>28</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>21</v>
@@ -2803,7 +2927,7 @@
         <v>39</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>13</v>
@@ -2831,7 +2955,7 @@
         <v>131</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>184</v>
@@ -2856,10 +2980,10 @@
         <v>220</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>131</v>
+        <v>39</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>53</v>
@@ -2879,8 +3003,324 @@
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
     </row>
+    <row r="66" spans="1:10" ht="105" hidden="1">
+      <c r="A66" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H66" s="3">
+        <v>46217</v>
+      </c>
+      <c r="I66" s="1"/>
+      <c r="J66" s="1"/>
+    </row>
+    <row r="67" spans="1:10" ht="90" hidden="1">
+      <c r="A67" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H67" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I67" s="1"/>
+      <c r="J67" s="1"/>
+    </row>
+    <row r="68" spans="1:10" ht="90" hidden="1">
+      <c r="A68" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H68" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I68" s="1"/>
+      <c r="J68" s="1"/>
+    </row>
+    <row r="69" spans="1:10" ht="75" hidden="1">
+      <c r="A69" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H69" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I69" s="1"/>
+      <c r="J69" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="45" hidden="1">
+      <c r="A70" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H70" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
+    </row>
+    <row r="71" spans="1:10" ht="120" hidden="1">
+      <c r="A71" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H71" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I71" s="1"/>
+      <c r="J71" s="1"/>
+    </row>
+    <row r="72" spans="1:10" ht="60" hidden="1">
+      <c r="A72" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="H72" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I72" s="1"/>
+      <c r="J72" s="1"/>
+    </row>
+    <row r="73" spans="1:10" ht="60">
+      <c r="A73" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="H73" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I73" s="1"/>
+      <c r="J73" s="1"/>
+    </row>
+    <row r="74" spans="1:10" ht="75">
+      <c r="A74" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H74" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I74" s="1"/>
+      <c r="J74" s="1"/>
+    </row>
+    <row r="75" spans="1:10" ht="45">
+      <c r="A75" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="H75" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I75" s="1"/>
+      <c r="J75" s="1"/>
+    </row>
+    <row r="76" spans="1:10" ht="135">
+      <c r="A76" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="H76" s="3">
+        <v>46220</v>
+      </c>
+      <c r="I76" s="1"/>
+      <c r="J76" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J76" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Open"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>